<commit_message>
regen all RE, fix modules to block
</commit_message>
<xml_diff>
--- a/БД/db/hwdb/А004.xlsx
+++ b/БД/db/hwdb/А004.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="28260" windowHeight="12360" activeTab="2"/>
+    <workbookView xWindow="120" yWindow="105" windowWidth="28260" windowHeight="12360" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Controls" sheetId="4" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="167">
   <si>
     <t>Modbus RTU</t>
   </si>
@@ -268,12 +268,6 @@
     <t>Модуль</t>
   </si>
   <si>
-    <t>Отказ модуля</t>
-  </si>
-  <si>
-    <t>Модуль не определен</t>
-  </si>
-  <si>
     <t>GENRBRF1_Top</t>
   </si>
   <si>
@@ -490,9 +484,6 @@
     <t>А004</t>
   </si>
   <si>
-    <t>Модуль сопряжения</t>
-  </si>
-  <si>
     <t>ТокВ1</t>
   </si>
   <si>
@@ -515,6 +506,18 @@
   </si>
   <si>
     <t>Измерительный токовый вход 4</t>
+  </si>
+  <si>
+    <t>Блок сопряжения</t>
+  </si>
+  <si>
+    <t>Отказ блока</t>
+  </si>
+  <si>
+    <t>Блок не определен</t>
+  </si>
+  <si>
+    <t>Блок</t>
   </si>
 </sst>
 </file>
@@ -856,14 +859,14 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1264,15 +1267,15 @@
       <c r="AW1" s="6"/>
       <c r="AX1" s="6"/>
       <c r="AY1" s="9"/>
-      <c r="AZ1" s="60" t="s">
+      <c r="AZ1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="BA1" s="61"/>
-      <c r="BB1" s="61"/>
-      <c r="BC1" s="61"/>
-      <c r="BD1" s="61"/>
-      <c r="BE1" s="61"/>
-      <c r="BF1" s="61"/>
+      <c r="BA1" s="62"/>
+      <c r="BB1" s="62"/>
+      <c r="BC1" s="62"/>
+      <c r="BD1" s="62"/>
+      <c r="BE1" s="62"/>
+      <c r="BF1" s="62"/>
     </row>
     <row r="2" spans="1:16379" s="17" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -25870,15 +25873,15 @@
       <c r="AW1" s="6"/>
       <c r="AX1" s="6"/>
       <c r="AY1" s="9"/>
-      <c r="AZ1" s="60" t="s">
+      <c r="AZ1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="BA1" s="61"/>
-      <c r="BB1" s="61"/>
-      <c r="BC1" s="61"/>
-      <c r="BD1" s="61"/>
-      <c r="BE1" s="61"/>
-      <c r="BF1" s="61"/>
+      <c r="BA1" s="62"/>
+      <c r="BB1" s="62"/>
+      <c r="BC1" s="62"/>
+      <c r="BD1" s="62"/>
+      <c r="BE1" s="62"/>
+      <c r="BF1" s="62"/>
     </row>
     <row r="2" spans="1:16379" s="17" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -42384,25 +42387,25 @@
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="30" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="H3" s="9"/>
       <c r="I3" s="20">
         <f t="shared" ref="I3:I4" si="0">LEN(F3)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J3" s="20" t="str">
         <f t="shared" ref="J3:J4" si="1">IF(LEN(F3)&lt;=$J$1,F3,"")</f>
-        <v>Отказ модуля</v>
+        <v>Отказ блока</v>
       </c>
       <c r="K3" s="24" t="s">
         <v>64</v>
@@ -42496,7 +42499,7 @@
       <c r="BF3" s="23"/>
       <c r="BG3" s="21" t="str">
         <f t="shared" ref="BG3:BG4" si="2">CONCATENATE("description: """,F3,"""", ", ", "note: """,E3,"""",", ","group: """, B3, """",", ","minValue: ", S3,", ","maxValue: ", T3,", ","step: ", U3,", ","units: """, R3, """",", ","defaultValue: ", X3,", ","eventRegistration: ", Y3,)</f>
-        <v>description: "Отказ модуля", note: "Отказ модуля", group: "status", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 2</v>
+        <v>description: "Отказ блока", note: "Отказ блока", group: "status", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 2</v>
       </c>
     </row>
     <row r="4" spans="1:16379" s="27" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -42506,25 +42509,25 @@
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="30" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>84</v>
+        <v>165</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>84</v>
+        <v>165</v>
       </c>
       <c r="H4" s="9"/>
       <c r="I4" s="20">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J4" s="20" t="str">
         <f t="shared" si="1"/>
-        <v>Модуль не определен</v>
+        <v>Блок не определен</v>
       </c>
       <c r="K4" s="24" t="s">
         <v>65</v>
@@ -42618,7 +42621,7 @@
       <c r="BF4" s="23"/>
       <c r="BG4" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>description: "Модуль не определен", note: "Критическая ошибка", group: "status", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 2</v>
+        <v>description: "Блок не определен", note: "Критическая ошибка", group: "status", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 2</v>
       </c>
     </row>
     <row r="5" spans="1:16379" s="27" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -42628,16 +42631,16 @@
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="30" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H5" s="9"/>
       <c r="I5" s="20">
@@ -42750,16 +42753,16 @@
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="30" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H6" s="9"/>
       <c r="I6" s="20">
@@ -42872,16 +42875,16 @@
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="30" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H7" s="9"/>
       <c r="I7" s="20">
@@ -42994,16 +42997,16 @@
       </c>
       <c r="C8" s="23"/>
       <c r="D8" s="30" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H8" s="9"/>
       <c r="I8" s="20">
@@ -50390,15 +50393,15 @@
       <c r="AW1" s="6"/>
       <c r="AX1" s="6"/>
       <c r="AY1" s="9"/>
-      <c r="AZ1" s="60" t="s">
+      <c r="AZ1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="BA1" s="61"/>
-      <c r="BB1" s="61"/>
-      <c r="BC1" s="61"/>
-      <c r="BD1" s="61"/>
-      <c r="BE1" s="61"/>
-      <c r="BF1" s="61"/>
+      <c r="BA1" s="62"/>
+      <c r="BB1" s="62"/>
+      <c r="BC1" s="62"/>
+      <c r="BD1" s="62"/>
+      <c r="BE1" s="62"/>
+      <c r="BF1" s="62"/>
     </row>
     <row r="2" spans="1:16379" s="17" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -66904,16 +66907,16 @@
       </c>
       <c r="C3" s="47"/>
       <c r="D3" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E3" s="48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F3" s="48" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G3" s="48" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H3" s="48"/>
       <c r="I3" s="48">
@@ -66925,10 +66928,10 @@
         <v/>
       </c>
       <c r="K3" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L3" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M3" s="47" t="s">
         <v>52</v>
@@ -66941,7 +66944,7 @@
         <v>2</v>
       </c>
       <c r="Q3" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R3" s="47" t="s">
         <v>53</v>
@@ -66981,23 +66984,23 @@
         <v>0</v>
       </c>
       <c r="AI3" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ3" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK3" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ3" s="53" t="s">
+      <c r="AL3" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK3" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL3" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM3" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN3" s="53"/>
       <c r="AO3" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP3" s="57" t="str">
         <f t="shared" ref="AP3:AP11" si="2">CONCATENATE(AJ3, ".", AL3)</f>
@@ -67044,16 +67047,16 @@
       </c>
       <c r="C4" s="47"/>
       <c r="D4" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E4" s="48" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F4" s="48" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G4" s="48" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H4" s="48"/>
       <c r="I4" s="48">
@@ -67065,10 +67068,10 @@
         <v/>
       </c>
       <c r="K4" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L4" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M4" s="47" t="s">
         <v>52</v>
@@ -67081,7 +67084,7 @@
         <v>2</v>
       </c>
       <c r="Q4" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R4" s="47" t="s">
         <v>53</v>
@@ -67121,23 +67124,23 @@
         <v>0</v>
       </c>
       <c r="AI4" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ4" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK4" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ4" s="53" t="s">
+      <c r="AL4" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK4" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL4" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM4" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN4" s="53"/>
       <c r="AO4" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP4" s="57" t="str">
         <f t="shared" si="2"/>
@@ -67184,16 +67187,16 @@
       </c>
       <c r="C5" s="47"/>
       <c r="D5" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E5" s="48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F5" s="48" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G5" s="48" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H5" s="48"/>
       <c r="I5" s="48">
@@ -67205,10 +67208,10 @@
         <v/>
       </c>
       <c r="K5" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L5" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M5" s="47" t="s">
         <v>52</v>
@@ -67221,7 +67224,7 @@
         <v>2</v>
       </c>
       <c r="Q5" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R5" s="47" t="s">
         <v>53</v>
@@ -67261,23 +67264,23 @@
         <v>0</v>
       </c>
       <c r="AI5" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ5" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK5" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ5" s="53" t="s">
+      <c r="AL5" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK5" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL5" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM5" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN5" s="53"/>
       <c r="AO5" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP5" s="57" t="str">
         <f t="shared" si="2"/>
@@ -67324,16 +67327,16 @@
       </c>
       <c r="C6" s="47"/>
       <c r="D6" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F6" s="48" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G6" s="48" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H6" s="48"/>
       <c r="I6" s="48">
@@ -67345,10 +67348,10 @@
         <v/>
       </c>
       <c r="K6" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L6" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M6" s="47" t="s">
         <v>52</v>
@@ -67361,7 +67364,7 @@
         <v>2</v>
       </c>
       <c r="Q6" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R6" s="47" t="s">
         <v>53</v>
@@ -67401,23 +67404,23 @@
         <v>0</v>
       </c>
       <c r="AI6" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ6" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK6" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ6" s="53" t="s">
+      <c r="AL6" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK6" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL6" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM6" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN6" s="53"/>
       <c r="AO6" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP6" s="57" t="str">
         <f t="shared" si="2"/>
@@ -67464,16 +67467,16 @@
       </c>
       <c r="C7" s="47"/>
       <c r="D7" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E7" s="48" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F7" s="48" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G7" s="48" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H7" s="48"/>
       <c r="I7" s="48">
@@ -67485,10 +67488,10 @@
         <v/>
       </c>
       <c r="K7" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L7" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M7" s="47" t="s">
         <v>52</v>
@@ -67501,19 +67504,19 @@
         <v>2</v>
       </c>
       <c r="Q7" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R7" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S7" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T7" s="47">
         <v>1000000</v>
       </c>
       <c r="U7" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V7" s="47"/>
       <c r="W7" s="47"/>
@@ -67541,23 +67544,23 @@
         <v>0</v>
       </c>
       <c r="AI7" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ7" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK7" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ7" s="53" t="s">
+      <c r="AL7" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK7" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL7" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM7" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN7" s="53"/>
       <c r="AO7" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP7" s="57" t="str">
         <f t="shared" si="2"/>
@@ -67604,16 +67607,16 @@
       </c>
       <c r="C8" s="47"/>
       <c r="D8" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F8" s="48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G8" s="48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H8" s="48"/>
       <c r="I8" s="48">
@@ -67625,10 +67628,10 @@
         <v/>
       </c>
       <c r="K8" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L8" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M8" s="47" t="s">
         <v>52</v>
@@ -67641,19 +67644,19 @@
         <v>2</v>
       </c>
       <c r="Q8" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R8" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S8" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T8" s="47">
         <v>1000000</v>
       </c>
       <c r="U8" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V8" s="47"/>
       <c r="W8" s="47"/>
@@ -67681,23 +67684,23 @@
         <v>0</v>
       </c>
       <c r="AI8" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ8" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK8" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ8" s="53" t="s">
+      <c r="AL8" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK8" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL8" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM8" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN8" s="53"/>
       <c r="AO8" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP8" s="57" t="str">
         <f t="shared" si="2"/>
@@ -67744,16 +67747,16 @@
       </c>
       <c r="C9" s="47"/>
       <c r="D9" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E9" s="48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F9" s="48" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G9" s="48" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H9" s="48"/>
       <c r="I9" s="48">
@@ -67765,10 +67768,10 @@
         <v/>
       </c>
       <c r="K9" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L9" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M9" s="47" t="s">
         <v>52</v>
@@ -67781,19 +67784,19 @@
         <v>2</v>
       </c>
       <c r="Q9" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R9" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S9" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T9" s="47">
         <v>1000000</v>
       </c>
       <c r="U9" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V9" s="47"/>
       <c r="W9" s="47"/>
@@ -67821,23 +67824,23 @@
         <v>0</v>
       </c>
       <c r="AI9" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ9" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK9" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ9" s="53" t="s">
+      <c r="AL9" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK9" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL9" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM9" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN9" s="53"/>
       <c r="AO9" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP9" s="57" t="str">
         <f t="shared" si="2"/>
@@ -67884,16 +67887,16 @@
       </c>
       <c r="C10" s="47"/>
       <c r="D10" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E10" s="48" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F10" s="48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G10" s="48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H10" s="48"/>
       <c r="I10" s="48">
@@ -67905,10 +67908,10 @@
         <v/>
       </c>
       <c r="K10" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L10" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M10" s="47" t="s">
         <v>52</v>
@@ -67921,19 +67924,19 @@
         <v>2</v>
       </c>
       <c r="Q10" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R10" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S10" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T10" s="47">
         <v>1000000</v>
       </c>
       <c r="U10" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V10" s="47"/>
       <c r="W10" s="47"/>
@@ -67961,23 +67964,23 @@
         <v>0</v>
       </c>
       <c r="AI10" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ10" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK10" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ10" s="53" t="s">
+      <c r="AL10" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK10" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL10" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM10" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN10" s="53"/>
       <c r="AO10" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP10" s="57" t="str">
         <f t="shared" si="2"/>
@@ -68024,16 +68027,16 @@
       </c>
       <c r="C11" s="47"/>
       <c r="D11" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E11" s="48" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F11" s="48" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G11" s="48" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H11" s="48"/>
       <c r="I11" s="48">
@@ -68045,10 +68048,10 @@
         <v>Метод расчета 1</v>
       </c>
       <c r="K11" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L11" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M11" s="47" t="s">
         <v>52</v>
@@ -68061,7 +68064,7 @@
         <v>2</v>
       </c>
       <c r="Q11" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R11" s="47" t="s">
         <v>53</v>
@@ -68101,23 +68104,23 @@
         <v>0</v>
       </c>
       <c r="AI11" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ11" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK11" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ11" s="53" t="s">
+      <c r="AL11" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK11" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL11" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM11" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN11" s="53"/>
       <c r="AO11" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP11" s="57" t="str">
         <f t="shared" si="2"/>
@@ -68164,16 +68167,16 @@
       </c>
       <c r="C12" s="47"/>
       <c r="D12" s="59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E12" s="48" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F12" s="48" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G12" s="48" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H12" s="49"/>
       <c r="I12" s="48">
@@ -68188,7 +68191,7 @@
         <v>63</v>
       </c>
       <c r="L12" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M12" s="47" t="s">
         <v>52</v>
@@ -68202,7 +68205,7 @@
       </c>
       <c r="Q12" s="50"/>
       <c r="R12" s="47" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="S12" s="47">
         <v>0</v>
@@ -68215,7 +68218,7 @@
       </c>
       <c r="V12" s="47"/>
       <c r="W12" s="47"/>
-      <c r="X12" s="62" t="s">
+      <c r="X12" s="60" t="s">
         <v>53</v>
       </c>
       <c r="Y12" s="47">
@@ -68287,16 +68290,16 @@
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H13" s="20"/>
       <c r="I13" s="20">
@@ -68308,10 +68311,10 @@
         <v/>
       </c>
       <c r="K13" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L13" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M13" s="25" t="s">
         <v>52</v>
@@ -68324,7 +68327,7 @@
         <v>2</v>
       </c>
       <c r="Q13" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R13" s="25" t="s">
         <v>53</v>
@@ -68364,23 +68367,23 @@
         <v>0</v>
       </c>
       <c r="AI13" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ13" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK13" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ13" s="23" t="s">
+      <c r="AL13" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK13" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL13" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM13" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN13" s="23"/>
       <c r="AO13" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP13" s="26" t="str">
         <f t="shared" ref="AP13:AP21" si="5">CONCATENATE(AJ13, ".", AL13)</f>
@@ -68427,16 +68430,16 @@
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H14" s="20"/>
       <c r="I14" s="20">
@@ -68448,10 +68451,10 @@
         <v/>
       </c>
       <c r="K14" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L14" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M14" s="25" t="s">
         <v>52</v>
@@ -68464,7 +68467,7 @@
         <v>2</v>
       </c>
       <c r="Q14" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R14" s="25" t="s">
         <v>53</v>
@@ -68504,23 +68507,23 @@
         <v>0</v>
       </c>
       <c r="AI14" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ14" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK14" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ14" s="23" t="s">
+      <c r="AL14" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK14" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL14" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM14" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN14" s="23"/>
       <c r="AO14" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP14" s="26" t="str">
         <f t="shared" si="5"/>
@@ -68567,16 +68570,16 @@
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H15" s="20"/>
       <c r="I15" s="20">
@@ -68588,10 +68591,10 @@
         <v/>
       </c>
       <c r="K15" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L15" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M15" s="25" t="s">
         <v>52</v>
@@ -68604,7 +68607,7 @@
         <v>2</v>
       </c>
       <c r="Q15" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R15" s="25" t="s">
         <v>53</v>
@@ -68644,23 +68647,23 @@
         <v>0</v>
       </c>
       <c r="AI15" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ15" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK15" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ15" s="23" t="s">
+      <c r="AL15" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK15" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL15" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM15" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN15" s="23"/>
       <c r="AO15" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP15" s="26" t="str">
         <f t="shared" si="5"/>
@@ -68707,16 +68710,16 @@
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H16" s="20"/>
       <c r="I16" s="20">
@@ -68728,10 +68731,10 @@
         <v/>
       </c>
       <c r="K16" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L16" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M16" s="25" t="s">
         <v>52</v>
@@ -68744,7 +68747,7 @@
         <v>2</v>
       </c>
       <c r="Q16" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R16" s="25" t="s">
         <v>53</v>
@@ -68784,23 +68787,23 @@
         <v>0</v>
       </c>
       <c r="AI16" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ16" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK16" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ16" s="23" t="s">
+      <c r="AL16" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK16" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL16" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM16" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN16" s="23"/>
       <c r="AO16" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP16" s="26" t="str">
         <f t="shared" si="5"/>
@@ -68847,16 +68850,16 @@
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H17" s="20"/>
       <c r="I17" s="20">
@@ -68868,10 +68871,10 @@
         <v/>
       </c>
       <c r="K17" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L17" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M17" s="25" t="s">
         <v>52</v>
@@ -68884,19 +68887,19 @@
         <v>2</v>
       </c>
       <c r="Q17" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R17" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S17" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T17" s="25">
         <v>1000000</v>
       </c>
       <c r="U17" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V17" s="25"/>
       <c r="W17" s="25"/>
@@ -68924,23 +68927,23 @@
         <v>0</v>
       </c>
       <c r="AI17" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ17" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK17" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ17" s="23" t="s">
+      <c r="AL17" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK17" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL17" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM17" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN17" s="23"/>
       <c r="AO17" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP17" s="26" t="str">
         <f t="shared" si="5"/>
@@ -68987,16 +68990,16 @@
       </c>
       <c r="C18" s="25"/>
       <c r="D18" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H18" s="20"/>
       <c r="I18" s="20">
@@ -69008,10 +69011,10 @@
         <v/>
       </c>
       <c r="K18" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L18" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M18" s="25" t="s">
         <v>52</v>
@@ -69024,19 +69027,19 @@
         <v>2</v>
       </c>
       <c r="Q18" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R18" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S18" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T18" s="25">
         <v>1000000</v>
       </c>
       <c r="U18" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V18" s="25"/>
       <c r="W18" s="25"/>
@@ -69064,23 +69067,23 @@
         <v>0</v>
       </c>
       <c r="AI18" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ18" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK18" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ18" s="23" t="s">
+      <c r="AL18" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK18" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL18" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM18" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN18" s="23"/>
       <c r="AO18" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP18" s="26" t="str">
         <f t="shared" si="5"/>
@@ -69127,16 +69130,16 @@
       </c>
       <c r="C19" s="25"/>
       <c r="D19" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H19" s="20"/>
       <c r="I19" s="20">
@@ -69148,10 +69151,10 @@
         <v/>
       </c>
       <c r="K19" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L19" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M19" s="25" t="s">
         <v>52</v>
@@ -69164,19 +69167,19 @@
         <v>2</v>
       </c>
       <c r="Q19" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R19" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S19" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T19" s="25">
         <v>1000000</v>
       </c>
       <c r="U19" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V19" s="25"/>
       <c r="W19" s="25"/>
@@ -69204,23 +69207,23 @@
         <v>0</v>
       </c>
       <c r="AI19" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ19" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK19" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ19" s="23" t="s">
+      <c r="AL19" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK19" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL19" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM19" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN19" s="23"/>
       <c r="AO19" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP19" s="26" t="str">
         <f t="shared" si="5"/>
@@ -69267,16 +69270,16 @@
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H20" s="20"/>
       <c r="I20" s="20">
@@ -69288,10 +69291,10 @@
         <v/>
       </c>
       <c r="K20" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L20" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M20" s="25" t="s">
         <v>52</v>
@@ -69304,19 +69307,19 @@
         <v>2</v>
       </c>
       <c r="Q20" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R20" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S20" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T20" s="25">
         <v>1000000</v>
       </c>
       <c r="U20" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V20" s="25"/>
       <c r="W20" s="25"/>
@@ -69344,23 +69347,23 @@
         <v>0</v>
       </c>
       <c r="AI20" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ20" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK20" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ20" s="23" t="s">
+      <c r="AL20" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK20" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL20" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM20" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN20" s="23"/>
       <c r="AO20" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP20" s="26" t="str">
         <f t="shared" si="5"/>
@@ -69407,16 +69410,16 @@
       </c>
       <c r="C21" s="25"/>
       <c r="D21" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H21" s="20"/>
       <c r="I21" s="20">
@@ -69428,10 +69431,10 @@
         <v>Метод расчета 2</v>
       </c>
       <c r="K21" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L21" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M21" s="25" t="s">
         <v>52</v>
@@ -69444,7 +69447,7 @@
         <v>2</v>
       </c>
       <c r="Q21" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R21" s="25" t="s">
         <v>53</v>
@@ -69484,23 +69487,23 @@
         <v>0</v>
       </c>
       <c r="AI21" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ21" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK21" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ21" s="23" t="s">
+      <c r="AL21" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK21" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL21" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM21" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN21" s="23"/>
       <c r="AO21" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP21" s="26" t="str">
         <f t="shared" si="5"/>
@@ -69547,16 +69550,16 @@
       </c>
       <c r="C22" s="25"/>
       <c r="D22" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H22" s="44"/>
       <c r="I22" s="20">
@@ -69571,7 +69574,7 @@
         <v>63</v>
       </c>
       <c r="L22" s="45" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M22" s="25" t="s">
         <v>52</v>
@@ -69585,7 +69588,7 @@
       </c>
       <c r="Q22" s="35"/>
       <c r="R22" s="25" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="S22" s="25">
         <v>0</v>
@@ -69598,7 +69601,7 @@
       </c>
       <c r="V22" s="25"/>
       <c r="W22" s="25"/>
-      <c r="X22" s="62" t="s">
+      <c r="X22" s="60" t="s">
         <v>53</v>
       </c>
       <c r="Y22" s="25">
@@ -69670,16 +69673,16 @@
       </c>
       <c r="C23" s="47"/>
       <c r="D23" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E23" s="48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F23" s="48" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G23" s="48" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H23" s="48"/>
       <c r="I23" s="48">
@@ -69691,10 +69694,10 @@
         <v/>
       </c>
       <c r="K23" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L23" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M23" s="47" t="s">
         <v>52</v>
@@ -69707,7 +69710,7 @@
         <v>2</v>
       </c>
       <c r="Q23" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R23" s="47" t="s">
         <v>53</v>
@@ -69747,23 +69750,23 @@
         <v>0</v>
       </c>
       <c r="AI23" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ23" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK23" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ23" s="53" t="s">
+      <c r="AL23" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK23" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL23" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM23" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN23" s="53"/>
       <c r="AO23" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP23" s="57" t="str">
         <f t="shared" ref="AP23:AP31" si="6">CONCATENATE(AJ23, ".", AL23)</f>
@@ -69810,16 +69813,16 @@
       </c>
       <c r="C24" s="47"/>
       <c r="D24" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E24" s="48" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F24" s="48" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G24" s="48" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H24" s="48"/>
       <c r="I24" s="48">
@@ -69831,10 +69834,10 @@
         <v/>
       </c>
       <c r="K24" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L24" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M24" s="47" t="s">
         <v>52</v>
@@ -69847,7 +69850,7 @@
         <v>2</v>
       </c>
       <c r="Q24" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R24" s="47" t="s">
         <v>53</v>
@@ -69887,23 +69890,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ24" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK24" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ24" s="53" t="s">
+      <c r="AL24" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK24" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL24" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM24" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN24" s="53"/>
       <c r="AO24" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP24" s="57" t="str">
         <f t="shared" si="6"/>
@@ -69950,16 +69953,16 @@
       </c>
       <c r="C25" s="47"/>
       <c r="D25" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E25" s="48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F25" s="48" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G25" s="48" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H25" s="48"/>
       <c r="I25" s="48">
@@ -69971,10 +69974,10 @@
         <v/>
       </c>
       <c r="K25" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L25" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M25" s="47" t="s">
         <v>52</v>
@@ -69987,7 +69990,7 @@
         <v>2</v>
       </c>
       <c r="Q25" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R25" s="47" t="s">
         <v>53</v>
@@ -70027,23 +70030,23 @@
         <v>0</v>
       </c>
       <c r="AI25" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ25" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK25" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ25" s="53" t="s">
+      <c r="AL25" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK25" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL25" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM25" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN25" s="53"/>
       <c r="AO25" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP25" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70090,16 +70093,16 @@
       </c>
       <c r="C26" s="47"/>
       <c r="D26" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E26" s="48" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F26" s="48" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G26" s="48" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H26" s="48"/>
       <c r="I26" s="48">
@@ -70111,10 +70114,10 @@
         <v/>
       </c>
       <c r="K26" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L26" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M26" s="47" t="s">
         <v>52</v>
@@ -70127,7 +70130,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R26" s="47" t="s">
         <v>53</v>
@@ -70167,23 +70170,23 @@
         <v>0</v>
       </c>
       <c r="AI26" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ26" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK26" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ26" s="53" t="s">
+      <c r="AL26" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK26" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL26" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM26" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN26" s="53"/>
       <c r="AO26" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP26" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70230,16 +70233,16 @@
       </c>
       <c r="C27" s="47"/>
       <c r="D27" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E27" s="48" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F27" s="48" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G27" s="48" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H27" s="48"/>
       <c r="I27" s="48">
@@ -70251,10 +70254,10 @@
         <v/>
       </c>
       <c r="K27" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L27" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M27" s="47" t="s">
         <v>52</v>
@@ -70267,19 +70270,19 @@
         <v>2</v>
       </c>
       <c r="Q27" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R27" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S27" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T27" s="47">
         <v>1000000</v>
       </c>
       <c r="U27" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V27" s="47"/>
       <c r="W27" s="47"/>
@@ -70307,23 +70310,23 @@
         <v>0</v>
       </c>
       <c r="AI27" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ27" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK27" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ27" s="53" t="s">
+      <c r="AL27" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK27" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL27" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM27" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN27" s="53"/>
       <c r="AO27" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP27" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70370,16 +70373,16 @@
       </c>
       <c r="C28" s="47"/>
       <c r="D28" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E28" s="48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F28" s="48" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G28" s="48" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H28" s="48"/>
       <c r="I28" s="48">
@@ -70391,10 +70394,10 @@
         <v/>
       </c>
       <c r="K28" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L28" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M28" s="47" t="s">
         <v>52</v>
@@ -70407,19 +70410,19 @@
         <v>2</v>
       </c>
       <c r="Q28" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R28" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S28" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T28" s="47">
         <v>1000000</v>
       </c>
       <c r="U28" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V28" s="47"/>
       <c r="W28" s="47"/>
@@ -70447,23 +70450,23 @@
         <v>0</v>
       </c>
       <c r="AI28" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ28" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK28" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ28" s="53" t="s">
+      <c r="AL28" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK28" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL28" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM28" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN28" s="53"/>
       <c r="AO28" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP28" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70510,16 +70513,16 @@
       </c>
       <c r="C29" s="47"/>
       <c r="D29" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E29" s="48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F29" s="48" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G29" s="48" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H29" s="48"/>
       <c r="I29" s="48">
@@ -70531,10 +70534,10 @@
         <v/>
       </c>
       <c r="K29" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L29" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M29" s="47" t="s">
         <v>52</v>
@@ -70547,19 +70550,19 @@
         <v>2</v>
       </c>
       <c r="Q29" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R29" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S29" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T29" s="47">
         <v>1000000</v>
       </c>
       <c r="U29" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V29" s="47"/>
       <c r="W29" s="47"/>
@@ -70587,23 +70590,23 @@
         <v>0</v>
       </c>
       <c r="AI29" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ29" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK29" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ29" s="53" t="s">
+      <c r="AL29" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK29" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL29" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM29" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN29" s="53"/>
       <c r="AO29" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP29" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70650,16 +70653,16 @@
       </c>
       <c r="C30" s="47"/>
       <c r="D30" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E30" s="48" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F30" s="48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G30" s="48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H30" s="48"/>
       <c r="I30" s="48">
@@ -70671,10 +70674,10 @@
         <v/>
       </c>
       <c r="K30" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L30" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M30" s="47" t="s">
         <v>52</v>
@@ -70687,19 +70690,19 @@
         <v>2</v>
       </c>
       <c r="Q30" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R30" s="47" t="s">
         <v>53</v>
       </c>
       <c r="S30" s="47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T30" s="47">
         <v>1000000</v>
       </c>
       <c r="U30" s="47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V30" s="47"/>
       <c r="W30" s="47"/>
@@ -70727,23 +70730,23 @@
         <v>0</v>
       </c>
       <c r="AI30" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ30" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK30" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ30" s="53" t="s">
+      <c r="AL30" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK30" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL30" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM30" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN30" s="53"/>
       <c r="AO30" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP30" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70790,16 +70793,16 @@
       </c>
       <c r="C31" s="47"/>
       <c r="D31" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E31" s="48" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F31" s="48" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G31" s="48" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H31" s="48"/>
       <c r="I31" s="48">
@@ -70811,10 +70814,10 @@
         <v>Метод расчета 3</v>
       </c>
       <c r="K31" s="46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L31" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M31" s="47" t="s">
         <v>52</v>
@@ -70827,7 +70830,7 @@
         <v>2</v>
       </c>
       <c r="Q31" s="50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R31" s="47" t="s">
         <v>53</v>
@@ -70867,23 +70870,23 @@
         <v>0</v>
       </c>
       <c r="AI31" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ31" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK31" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="AJ31" s="53" t="s">
+      <c r="AL31" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="AK31" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL31" s="53" t="s">
-        <v>91</v>
-      </c>
       <c r="AM31" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN31" s="53"/>
       <c r="AO31" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP31" s="57" t="str">
         <f t="shared" si="6"/>
@@ -70930,16 +70933,16 @@
       </c>
       <c r="C32" s="47"/>
       <c r="D32" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E32" s="48" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F32" s="48" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G32" s="48" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H32" s="49"/>
       <c r="I32" s="48">
@@ -70954,7 +70957,7 @@
         <v>63</v>
       </c>
       <c r="L32" s="56" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M32" s="47" t="s">
         <v>52</v>
@@ -70968,7 +70971,7 @@
       </c>
       <c r="Q32" s="50"/>
       <c r="R32" s="47" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="S32" s="47">
         <v>0</v>
@@ -70981,7 +70984,7 @@
       </c>
       <c r="V32" s="47"/>
       <c r="W32" s="47"/>
-      <c r="X32" s="62" t="s">
+      <c r="X32" s="60" t="s">
         <v>53</v>
       </c>
       <c r="Y32" s="47">
@@ -71053,16 +71056,16 @@
       </c>
       <c r="C33" s="25"/>
       <c r="D33" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F33" s="20" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G33" s="20" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H33" s="20"/>
       <c r="I33" s="20">
@@ -71074,10 +71077,10 @@
         <v/>
       </c>
       <c r="K33" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L33" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M33" s="25" t="s">
         <v>52</v>
@@ -71090,7 +71093,7 @@
         <v>2</v>
       </c>
       <c r="Q33" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R33" s="25" t="s">
         <v>53</v>
@@ -71130,23 +71133,23 @@
         <v>0</v>
       </c>
       <c r="AI33" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ33" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK33" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ33" s="23" t="s">
+      <c r="AL33" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK33" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL33" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM33" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN33" s="23"/>
       <c r="AO33" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP33" s="26" t="str">
         <f t="shared" ref="AP33:AP41" si="7">CONCATENATE(AJ33, ".", AL33)</f>
@@ -71193,16 +71196,16 @@
       </c>
       <c r="C34" s="25"/>
       <c r="D34" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E34" s="20" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F34" s="20" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H34" s="20"/>
       <c r="I34" s="20">
@@ -71214,10 +71217,10 @@
         <v/>
       </c>
       <c r="K34" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L34" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M34" s="25" t="s">
         <v>52</v>
@@ -71230,7 +71233,7 @@
         <v>2</v>
       </c>
       <c r="Q34" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R34" s="25" t="s">
         <v>53</v>
@@ -71270,23 +71273,23 @@
         <v>0</v>
       </c>
       <c r="AI34" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ34" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK34" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ34" s="23" t="s">
+      <c r="AL34" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK34" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL34" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM34" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN34" s="23"/>
       <c r="AO34" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP34" s="26" t="str">
         <f t="shared" si="7"/>
@@ -71333,16 +71336,16 @@
       </c>
       <c r="C35" s="25"/>
       <c r="D35" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E35" s="20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H35" s="20"/>
       <c r="I35" s="20">
@@ -71354,10 +71357,10 @@
         <v/>
       </c>
       <c r="K35" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L35" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M35" s="25" t="s">
         <v>52</v>
@@ -71370,7 +71373,7 @@
         <v>2</v>
       </c>
       <c r="Q35" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R35" s="25" t="s">
         <v>53</v>
@@ -71410,23 +71413,23 @@
         <v>0</v>
       </c>
       <c r="AI35" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ35" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK35" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ35" s="23" t="s">
+      <c r="AL35" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK35" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL35" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM35" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN35" s="23"/>
       <c r="AO35" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP35" s="26" t="str">
         <f t="shared" si="7"/>
@@ -71473,16 +71476,16 @@
       </c>
       <c r="C36" s="25"/>
       <c r="D36" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E36" s="20" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F36" s="20" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H36" s="20"/>
       <c r="I36" s="20">
@@ -71494,10 +71497,10 @@
         <v/>
       </c>
       <c r="K36" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L36" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M36" s="25" t="s">
         <v>52</v>
@@ -71510,7 +71513,7 @@
         <v>2</v>
       </c>
       <c r="Q36" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R36" s="25" t="s">
         <v>53</v>
@@ -71550,23 +71553,23 @@
         <v>0</v>
       </c>
       <c r="AI36" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ36" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK36" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ36" s="23" t="s">
+      <c r="AL36" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK36" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL36" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM36" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN36" s="23"/>
       <c r="AO36" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP36" s="26" t="str">
         <f t="shared" si="7"/>
@@ -71613,16 +71616,16 @@
       </c>
       <c r="C37" s="25"/>
       <c r="D37" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H37" s="20"/>
       <c r="I37" s="20">
@@ -71634,10 +71637,10 @@
         <v/>
       </c>
       <c r="K37" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L37" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M37" s="25" t="s">
         <v>52</v>
@@ -71650,19 +71653,19 @@
         <v>2</v>
       </c>
       <c r="Q37" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R37" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S37" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T37" s="25">
         <v>1000000</v>
       </c>
       <c r="U37" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V37" s="25"/>
       <c r="W37" s="25"/>
@@ -71690,23 +71693,23 @@
         <v>0</v>
       </c>
       <c r="AI37" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ37" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK37" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ37" s="23" t="s">
+      <c r="AL37" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK37" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL37" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM37" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN37" s="23"/>
       <c r="AO37" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP37" s="26" t="str">
         <f t="shared" si="7"/>
@@ -71753,16 +71756,16 @@
       </c>
       <c r="C38" s="25"/>
       <c r="D38" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E38" s="20" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F38" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G38" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H38" s="20"/>
       <c r="I38" s="20">
@@ -71774,10 +71777,10 @@
         <v/>
       </c>
       <c r="K38" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L38" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M38" s="25" t="s">
         <v>52</v>
@@ -71790,19 +71793,19 @@
         <v>2</v>
       </c>
       <c r="Q38" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R38" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S38" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T38" s="25">
         <v>1000000</v>
       </c>
       <c r="U38" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V38" s="25"/>
       <c r="W38" s="25"/>
@@ -71830,23 +71833,23 @@
         <v>0</v>
       </c>
       <c r="AI38" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ38" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK38" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ38" s="23" t="s">
+      <c r="AL38" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK38" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL38" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM38" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN38" s="23"/>
       <c r="AO38" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP38" s="26" t="str">
         <f t="shared" si="7"/>
@@ -71893,16 +71896,16 @@
       </c>
       <c r="C39" s="25"/>
       <c r="D39" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G39" s="20" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H39" s="20"/>
       <c r="I39" s="20">
@@ -71914,10 +71917,10 @@
         <v/>
       </c>
       <c r="K39" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L39" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M39" s="25" t="s">
         <v>52</v>
@@ -71930,19 +71933,19 @@
         <v>2</v>
       </c>
       <c r="Q39" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R39" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S39" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T39" s="25">
         <v>1000000</v>
       </c>
       <c r="U39" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V39" s="25"/>
       <c r="W39" s="25"/>
@@ -71970,23 +71973,23 @@
         <v>0</v>
       </c>
       <c r="AI39" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ39" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK39" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ39" s="23" t="s">
+      <c r="AL39" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK39" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL39" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM39" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN39" s="23"/>
       <c r="AO39" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP39" s="26" t="str">
         <f t="shared" si="7"/>
@@ -72033,16 +72036,16 @@
       </c>
       <c r="C40" s="25"/>
       <c r="D40" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G40" s="20" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H40" s="20"/>
       <c r="I40" s="20">
@@ -72054,10 +72057,10 @@
         <v/>
       </c>
       <c r="K40" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L40" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M40" s="25" t="s">
         <v>52</v>
@@ -72070,19 +72073,19 @@
         <v>2</v>
       </c>
       <c r="Q40" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R40" s="25" t="s">
         <v>53</v>
       </c>
       <c r="S40" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T40" s="25">
         <v>1000000</v>
       </c>
       <c r="U40" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="V40" s="25"/>
       <c r="W40" s="25"/>
@@ -72110,23 +72113,23 @@
         <v>0</v>
       </c>
       <c r="AI40" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ40" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK40" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ40" s="23" t="s">
+      <c r="AL40" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK40" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL40" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM40" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN40" s="23"/>
       <c r="AO40" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP40" s="26" t="str">
         <f t="shared" si="7"/>
@@ -72173,16 +72176,16 @@
       </c>
       <c r="C41" s="25"/>
       <c r="D41" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E41" s="20" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F41" s="20" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H41" s="20"/>
       <c r="I41" s="20">
@@ -72194,10 +72197,10 @@
         <v>Метод расчета 4</v>
       </c>
       <c r="K41" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L41" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M41" s="25" t="s">
         <v>52</v>
@@ -72210,7 +72213,7 @@
         <v>2</v>
       </c>
       <c r="Q41" s="35" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="R41" s="25" t="s">
         <v>53</v>
@@ -72250,23 +72253,23 @@
         <v>0</v>
       </c>
       <c r="AI41" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AJ41" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="AK41" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AJ41" s="23" t="s">
+      <c r="AL41" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AK41" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="AL41" s="23" t="s">
-        <v>91</v>
-      </c>
       <c r="AM41" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AN41" s="23"/>
       <c r="AO41" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AP41" s="26" t="str">
         <f t="shared" si="7"/>
@@ -72313,16 +72316,16 @@
       </c>
       <c r="C42" s="25"/>
       <c r="D42" s="30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E42" s="20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G42" s="20" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H42" s="44"/>
       <c r="I42" s="20">
@@ -72337,7 +72340,7 @@
         <v>63</v>
       </c>
       <c r="L42" s="45" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M42" s="25" t="s">
         <v>52</v>
@@ -72351,7 +72354,7 @@
       </c>
       <c r="Q42" s="35"/>
       <c r="R42" s="25" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="S42" s="25">
         <v>0</v>
@@ -72364,7 +72367,7 @@
       </c>
       <c r="V42" s="25"/>
       <c r="W42" s="25"/>
-      <c r="X42" s="62" t="s">
+      <c r="X42" s="60" t="s">
         <v>53</v>
       </c>
       <c r="Y42" s="25">
@@ -72461,7 +72464,7 @@
         <v>59</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -72485,7 +72488,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -72501,7 +72504,7 @@
         <v>76</v>
       </c>
       <c r="B8" s="41" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -72515,20 +72518,20 @@
         <v>82</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="58" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B11" s="58" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B12" s="40">
         <v>4</v>
@@ -72536,7 +72539,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="58" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B13" s="40">
         <v>0</v>
@@ -72544,34 +72547,34 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="58" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="58" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="58" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="58" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>